<commit_message>
bug report update v5
</commit_message>
<xml_diff>
--- a/test-cases/functional-test.xlsx
+++ b/test-cases/functional-test.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kiris\OneDrive\Desktop\senior-qa-case\test cases\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kiris\OneDrive\Desktop\senior-qa-case\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3410AD0F-75FB-416D-9AC5-3415DF87C413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE8FFF44-4028-43CF-B150-BD8FC0C3E7F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kullanıcı Kimlik Doğrulama" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1717" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1719" uniqueCount="345">
   <si>
     <t>TCID</t>
   </si>
@@ -1236,6 +1236,12 @@
   </si>
   <si>
     <t>BUG-015</t>
+  </si>
+  <si>
+    <t>Zorunluluk uyarısının çıkmadığı görüldü</t>
+  </si>
+  <si>
+    <t>BUG-016</t>
   </si>
 </sst>
 </file>
@@ -6642,7 +6648,7 @@
     <col min="7" max="7" width="120" style="9" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="93.84375" style="9" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="65.69140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.69140625" style="9" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.3046875" style="9" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="53.3046875" style="9" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="8.23046875" style="9" bestFit="1" customWidth="1"/>
     <col min="13" max="16384" width="9" style="9"/>
@@ -7198,13 +7204,17 @@
         <v>226</v>
       </c>
       <c r="I28" s="5" t="s">
-        <v>227</v>
-      </c>
-      <c r="J28" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="K28" s="4"/>
-      <c r="L28" s="4"/>
+        <v>343</v>
+      </c>
+      <c r="J28" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="K28" s="11" t="s">
+        <v>254</v>
+      </c>
+      <c r="L28" s="11" t="s">
+        <v>339</v>
+      </c>
     </row>
     <row r="29" spans="1:12" s="5" customFormat="1">
       <c r="F29" s="5">
@@ -7226,7 +7236,7 @@
         <v>254</v>
       </c>
       <c r="L29" s="11" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="30" spans="1:12" s="5" customFormat="1">
@@ -7575,7 +7585,7 @@
         <v>257</v>
       </c>
       <c r="L47" s="11" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="48" spans="1:12" s="5" customFormat="1">
@@ -7716,7 +7726,7 @@
         <v>257</v>
       </c>
       <c r="L54" s="11" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="55" spans="1:12" s="5" customFormat="1">
@@ -7857,7 +7867,7 @@
         <v>257</v>
       </c>
       <c r="L61" s="11" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="62" spans="1:12" s="5" customFormat="1">

</xml_diff>